<commit_message>
Updated iMoni test report templates
</commit_message>
<xml_diff>
--- a/server/ATS/template/green-pcb_allpassed_template.xlsx
+++ b/server/ATS/template/green-pcb_allpassed_template.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A5DB76-3885-4782-938D-73341F1E5504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09594748-43AC-404E-AECD-5992C646ADFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
   <si>
     <t>IMONI ASSEMBLY TEST REPORT</t>
   </si>
@@ -23,33 +23,12 @@
     <t>Report No:</t>
   </si>
   <si>
-    <t xml:space="preserve">Assembly Sr. No. </t>
-  </si>
-  <si>
     <t>DateTime:</t>
   </si>
   <si>
     <t>TestLevel:</t>
   </si>
   <si>
-    <t>iMoni Assembly</t>
-  </si>
-  <si>
-    <t>DeviceIP:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CPU Sr. No. </t>
-  </si>
-  <si>
-    <t>Base PCB Sr. No.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Camera Sr. No. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PSU Sr. No. </t>
-  </si>
-  <si>
     <t>TotalTests:</t>
   </si>
   <si>
@@ -104,49 +83,19 @@
     <t>EM Lock through Keypad</t>
   </si>
   <si>
-    <t>EM Lock through eMS</t>
-  </si>
-  <si>
     <t>Water Logging Test</t>
   </si>
   <si>
     <t>Humidity Test</t>
   </si>
   <si>
-    <t>Inside Temperature Test</t>
-  </si>
-  <si>
-    <t>Outside Temperature Test</t>
-  </si>
-  <si>
-    <t>Non - Critical Load Test</t>
-  </si>
-  <si>
-    <t>Camera Test</t>
-  </si>
-  <si>
-    <t>Fan-Fail Test Test</t>
-  </si>
-  <si>
-    <t>HUPS</t>
-  </si>
-  <si>
-    <t>iMoni-SRMS-0058</t>
-  </si>
-  <si>
-    <t>TTiMGPE26000K013</t>
-  </si>
-  <si>
-    <t>LB/F/26/9188</t>
-  </si>
-  <si>
     <t>OPERATOR:</t>
   </si>
   <si>
     <t>APPROVED BY:</t>
   </si>
   <si>
-    <t>192.168.0.49</t>
+    <t xml:space="preserve">PCB Serial No. </t>
   </si>
 </sst>
 </file>
@@ -170,7 +119,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -231,21 +180,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -321,21 +255,6 @@
     </border>
     <border>
       <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
@@ -503,64 +422,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -570,16 +493,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -899,7 +822,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" customWidth="1"/>
@@ -910,403 +833,253 @@
     <col min="6" max="6" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="31"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="26"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="4"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="B2" s="20"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="21"/>
+      <c r="F3" s="5"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="7"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="B4" s="22"/>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="8">
-        <v>46217.560590277775</v>
-      </c>
-      <c r="F4" s="7"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="B5" s="21"/>
+      <c r="F5" s="5"/>
+    </row>
+    <row r="6" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B6" s="23"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="19"/>
+    </row>
+    <row r="7" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="F7" s="5"/>
+    </row>
+    <row r="8" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="7"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="B8" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="9" t="s">
+      <c r="C8" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D8" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F8" s="12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="13">
+        <v>1</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="4">
+        <v>2</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="17"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
+        <v>3</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="6">
+        <v>9</v>
+      </c>
+      <c r="E11" s="16"/>
+      <c r="F11" s="17"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>4</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="6">
+        <v>3</v>
+      </c>
+      <c r="E12" s="16"/>
+      <c r="F12" s="17"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="13">
+        <v>5</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="6">
+        <v>3</v>
+      </c>
+      <c r="E13" s="16"/>
+      <c r="F13" s="17"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <v>6</v>
+      </c>
+      <c r="B14" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="12">
-        <v>16</v>
-      </c>
-      <c r="C7" s="25">
-        <v>49</v>
-      </c>
-      <c r="D7" s="25">
-        <v>59</v>
-      </c>
-      <c r="E7" s="25">
-        <v>32</v>
-      </c>
-      <c r="F7" s="26" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="15"/>
-      <c r="B8" s="16"/>
-      <c r="F8" s="7"/>
-    </row>
-    <row r="9" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="18" t="s">
+      <c r="C14" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="20">
+      <c r="D14" s="6">
+        <v>3</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="F14" s="17"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="13">
+        <v>7</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="6">
+        <v>3</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="F15" s="17"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
+        <v>8</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="6">
+        <v>3</v>
+      </c>
+      <c r="E16" s="16"/>
+      <c r="F16" s="17"/>
+    </row>
+    <row r="17" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="13">
+        <v>9</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="6">
         <v>1</v>
       </c>
-      <c r="B10" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="F10" s="22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="5">
-        <v>2</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23" t="s">
+      <c r="E17" s="16"/>
+      <c r="F17" s="17"/>
+    </row>
+    <row r="18" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="24"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="5">
-        <v>3</v>
-      </c>
-      <c r="B12" s="23" t="s">
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D12" s="9">
-        <v>9</v>
-      </c>
-      <c r="E12" s="23"/>
-      <c r="F12" s="24"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="5">
-        <v>4</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="9">
-        <v>3</v>
-      </c>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="5">
-        <v>5</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="9">
-        <v>3</v>
-      </c>
-      <c r="E14" s="23"/>
-      <c r="F14" s="24"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="5">
-        <v>6</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15" s="9">
-        <v>3</v>
-      </c>
-      <c r="E15" s="23"/>
-      <c r="F15" s="24"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="5">
-        <v>7</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="9">
-        <v>3</v>
-      </c>
-      <c r="E16" s="23"/>
-      <c r="F16" s="24"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="5">
-        <v>8</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17" s="9">
-        <v>3</v>
-      </c>
-      <c r="E17" s="23"/>
-      <c r="F17" s="24"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="5">
-        <v>9</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18" s="9">
-        <v>3</v>
-      </c>
-      <c r="E18" s="23"/>
-      <c r="F18" s="24"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="5">
-        <v>10</v>
-      </c>
-      <c r="B19" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="9">
-        <v>1</v>
-      </c>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="5">
-        <v>11</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D20" s="9">
-        <v>1</v>
-      </c>
-      <c r="E20" s="23"/>
-      <c r="F20" s="24"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="5">
-        <v>12</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C21" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D21" s="9">
-        <v>1</v>
-      </c>
-      <c r="E21" s="23"/>
-      <c r="F21" s="24"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="5">
-        <v>13</v>
-      </c>
-      <c r="B22" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D22" s="9">
-        <v>3</v>
-      </c>
-      <c r="E22" s="23"/>
-      <c r="F22" s="24"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="5">
-        <v>14</v>
-      </c>
-      <c r="B23" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="C23" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" s="9">
-        <v>1</v>
-      </c>
-      <c r="E23" s="23"/>
-      <c r="F23" s="24"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="5">
-        <v>15</v>
-      </c>
-      <c r="B24" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="9">
-        <v>2</v>
-      </c>
-      <c r="E24" s="23"/>
-      <c r="F24" s="24"/>
-    </row>
-    <row r="25" spans="1:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="11">
-        <v>16</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" s="25">
-        <v>1</v>
-      </c>
-      <c r="E25" s="13"/>
-      <c r="F25" s="14"/>
-    </row>
-    <row r="26" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="32" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="4"/>
-    </row>
-    <row r="27" spans="1:6" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="33"/>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="28"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="1:6" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="28"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="D18:D19"/>
   </mergeCells>
   <pageMargins left="0.19" right="0.19" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="98" orientation="portrait" useFirstPageNumber="1" horizontalDpi="1200" verticalDpi="1200"/>

</xml_diff>